<commit_message>
changes in area upload format
</commit_message>
<xml_diff>
--- a/uploads/excel_format/bulk upload format.xlsx
+++ b/uploads/excel_format/bulk upload format.xlsx
@@ -1,20 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Marudham\uploads\excel_format\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="139">
   <si>
     <t>Sl.no</t>
   </si>
@@ -65,9 +60,6 @@
     <t>area</t>
   </si>
   <si>
-    <t>sub_area</t>
-  </si>
-  <si>
     <t>address</t>
   </si>
   <si>
@@ -110,9 +102,6 @@
     <t>loan_category</t>
   </si>
   <si>
-    <t>sub_category</t>
-  </si>
-  <si>
     <t>tot_value</t>
   </si>
   <si>
@@ -339,9 +328,6 @@
   </si>
   <si>
     <t>Appliance</t>
-  </si>
-  <si>
-    <t>Electronics</t>
   </si>
   <si>
     <t>Due Amount</t>
@@ -456,8 +442,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-14009]yyyy/mm/dd;@"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -506,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -523,6 +510,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,7 +573,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -618,7 +608,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -795,7 +785,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -803,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CS13"/>
+  <dimension ref="A1:CQ13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
@@ -819,90 +809,88 @@
     <col min="11" max="11" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="17" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="10" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="18" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="11" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="21" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="11" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="14" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="8" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="11" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="78" max="79" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="18" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="12" bestFit="1" customWidth="1"/>
-    <col min="88" max="88" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="89" max="89" width="14" bestFit="1" customWidth="1"/>
-    <col min="90" max="90" width="6" bestFit="1" customWidth="1"/>
-    <col min="91" max="91" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="93" max="93" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="94" max="94" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="95" max="96" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="39.85546875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="18" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="11" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="21" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="11" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="14" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="8" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="11" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="76" max="77" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="18" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="12" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="14" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="6" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="91" max="91" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="93" max="94" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:97" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:95" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -1102,13 +1090,13 @@
         <v>65</v>
       </c>
       <c r="BO1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="BP1" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" s="9" t="s">
+      <c r="BQ1" s="9" t="s">
         <v>67</v>
-      </c>
-      <c r="BQ1" s="9" t="s">
-        <v>34</v>
       </c>
       <c r="BR1" s="9" t="s">
         <v>68</v>
@@ -1177,308 +1165,296 @@
         <v>89</v>
       </c>
       <c r="CN1" s="9" t="s">
-        <v>90</v>
+        <v>129</v>
       </c>
       <c r="CO1" s="9" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="CP1" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="CQ1" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="CR1" s="9" t="s">
-        <v>134</v>
-      </c>
-      <c r="CS1" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
-    <row r="2" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="10">
         <v>45238</v>
       </c>
       <c r="C2" s="3">
         <v>271232712327</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="G2" s="2">
+        <v>136</v>
+      </c>
+      <c r="G2" s="10">
         <v>32874</v>
       </c>
       <c r="H2" s="4">
         <v>34</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="M2" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="N2" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="O2" s="1">
+        <v>2712327123</v>
+      </c>
+      <c r="P2" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="Q2" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="N2" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="P2" s="1">
-        <v>2712327123</v>
-      </c>
-      <c r="Q2" s="5" t="s">
+      <c r="R2" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="S2" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="T2" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="V2" s="3">
+        <v>111111111111</v>
+      </c>
+      <c r="W2" s="4">
+        <v>30</v>
+      </c>
+      <c r="X2" s="1">
+        <v>8124222132</v>
+      </c>
+      <c r="Y2" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="U2" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="Z2" s="1">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="W2" s="3">
-        <v>111111111111</v>
-      </c>
-      <c r="X2" s="4">
-        <v>30</v>
-      </c>
-      <c r="Y2" s="1">
-        <v>8124222132</v>
-      </c>
-      <c r="Z2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="AA2" s="1">
+      <c r="AB2" s="1">
+        <v>15000</v>
+      </c>
+      <c r="AC2" s="1">
         <v>0</v>
-      </c>
-      <c r="AB2" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="AC2" s="6" t="s">
-        <v>105</v>
       </c>
       <c r="AD2" s="1">
         <v>15000</v>
       </c>
-      <c r="AE2" s="1">
+      <c r="AE2" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="AF2" s="1">
+        <v>2800</v>
+      </c>
+      <c r="AG2" s="4"/>
+      <c r="AH2" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="AI2" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="AJ2" s="4"/>
+      <c r="AK2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AL2" s="1">
         <v>0</v>
       </c>
-      <c r="AF2" s="1">
-        <v>15000</v>
-      </c>
-      <c r="AG2" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AH2" s="1">
-        <v>2800</v>
-      </c>
-      <c r="AI2" s="4"/>
-      <c r="AJ2" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="AK2" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="AL2" s="4"/>
-      <c r="AM2" s="1" t="s">
-        <v>109</v>
+      <c r="AM2" s="1">
+        <v>0</v>
       </c>
       <c r="AN2" s="1">
         <v>0</v>
       </c>
       <c r="AO2" s="1">
-        <v>0</v>
+        <v>32000</v>
       </c>
       <c r="AP2" s="1">
         <v>0</v>
       </c>
       <c r="AQ2" s="1">
-        <v>32000</v>
+        <v>0</v>
       </c>
       <c r="AR2" s="1">
         <v>0</v>
       </c>
       <c r="AS2" s="1">
+        <v>5000</v>
+      </c>
+      <c r="AT2" s="1">
+        <v>100000</v>
+      </c>
+      <c r="AU2" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="AV2" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="AW2" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="AX2" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="AY2" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="AZ2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="BA2" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="BB2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BC2" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="BD2" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="BE2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="BF2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="BG2" s="10">
+        <v>45238</v>
+      </c>
+      <c r="BH2" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="BI2" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="BJ2" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="BK2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="BL2" s="4"/>
+      <c r="BM2" s="4"/>
+      <c r="BN2" s="1">
+        <v>2</v>
+      </c>
+      <c r="BO2" s="1">
+        <v>6</v>
+      </c>
+      <c r="BP2" s="4">
+        <v>2</v>
+      </c>
+      <c r="BQ2" s="1">
         <v>0</v>
       </c>
-      <c r="AT2" s="1">
+      <c r="BR2" s="1">
+        <v>15000</v>
+      </c>
+      <c r="BS2" s="1">
+        <v>15000</v>
+      </c>
+      <c r="BT2" s="7">
+        <v>1800</v>
+      </c>
+      <c r="BU2" s="7">
+        <v>16800</v>
+      </c>
+      <c r="BV2" s="1">
+        <v>2800</v>
+      </c>
+      <c r="BW2" s="7">
+        <v>300</v>
+      </c>
+      <c r="BX2" s="4">
         <v>0</v>
       </c>
-      <c r="AU2" s="1">
-        <v>5000</v>
-      </c>
-      <c r="AV2" s="1">
-        <v>100000</v>
-      </c>
-      <c r="AW2" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="AX2" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="AY2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="AZ2" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="BA2" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BB2" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="BC2" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="BD2" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="BE2" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="BF2" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="BG2" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="BH2" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="BI2" s="2">
-        <v>45238</v>
-      </c>
-      <c r="BJ2" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="BK2" s="1" t="s">
+      <c r="BY2" s="7">
+        <v>14700</v>
+      </c>
+      <c r="BZ2" s="10">
+        <v>45270</v>
+      </c>
+      <c r="CA2" s="10">
+        <v>45422</v>
+      </c>
+      <c r="CB2" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="BL2" s="1" t="s">
+      <c r="CC2" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="BM2" s="1" t="s">
+      <c r="CD2" s="3">
+        <v>239903777436</v>
+      </c>
+      <c r="CE2" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="BN2" s="4"/>
-      <c r="BO2" s="4"/>
-      <c r="BP2" s="1">
-        <v>2</v>
-      </c>
-      <c r="BQ2" s="1">
-        <v>6</v>
-      </c>
-      <c r="BR2" s="4">
-        <v>2</v>
-      </c>
-      <c r="BS2" s="1">
+      <c r="CF2" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="CG2" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="CH2" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="CI2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="CJ2" s="7">
+        <v>14700</v>
+      </c>
+      <c r="CK2" s="4">
         <v>0</v>
       </c>
-      <c r="BT2" s="1">
-        <v>15000</v>
-      </c>
-      <c r="BU2" s="1">
-        <v>15000</v>
-      </c>
-      <c r="BV2" s="7">
-        <v>1800</v>
-      </c>
-      <c r="BW2" s="7">
-        <v>16800</v>
-      </c>
-      <c r="BX2" s="1">
-        <v>2800</v>
-      </c>
-      <c r="BY2" s="7">
-        <v>300</v>
-      </c>
-      <c r="BZ2" s="4">
-        <v>0</v>
-      </c>
-      <c r="CA2" s="7">
-        <v>14700</v>
-      </c>
-      <c r="CB2" s="2">
-        <v>45270</v>
-      </c>
-      <c r="CC2" s="2">
-        <v>45422</v>
-      </c>
-      <c r="CD2" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="CE2" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="CF2" s="3">
+      <c r="CL2" s="3">
         <v>239903777436</v>
       </c>
-      <c r="CG2" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="CH2" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="CI2" s="6" t="s">
+      <c r="CM2" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="CJ2" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="CK2" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="CL2" s="7">
-        <v>14700</v>
-      </c>
-      <c r="CM2" s="4">
-        <v>0</v>
-      </c>
-      <c r="CN2" s="3">
-        <v>239903777436</v>
-      </c>
-      <c r="CO2" s="1" t="s">
-        <v>128</v>
+      <c r="CN2" t="s">
+        <v>132</v>
+      </c>
+      <c r="CO2" t="s">
+        <v>133</v>
       </c>
       <c r="CP2" t="s">
-        <v>135</v>
-      </c>
-      <c r="CQ2" t="s">
-        <v>136</v>
-      </c>
-      <c r="CR2" t="s">
-        <v>137</v>
-      </c>
-      <c r="CS2" s="2">
+        <v>134</v>
+      </c>
+      <c r="CQ2" s="2">
         <v>45483</v>
       </c>
     </row>
-    <row r="3" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" s="3"/>
@@ -1492,31 +1468,31 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="8"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="1"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="8"/>
       <c r="T3" s="8"/>
-      <c r="U3" s="8"/>
-      <c r="V3" s="1"/>
-      <c r="W3" s="3"/>
-      <c r="X3" s="4"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
-      <c r="AA3" s="1"/>
-      <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="1"/>
+      <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
       <c r="AE3" s="1"/>
       <c r="AF3" s="1"/>
-      <c r="AG3" s="1"/>
-      <c r="AH3" s="1"/>
-      <c r="AI3" s="4"/>
-      <c r="AJ3" s="8"/>
-      <c r="AK3" s="8"/>
-      <c r="AL3" s="4"/>
+      <c r="AG3" s="4"/>
+      <c r="AH3" s="8"/>
+      <c r="AI3" s="8"/>
+      <c r="AJ3" s="4"/>
+      <c r="AK3" s="1"/>
+      <c r="AL3" s="1"/>
       <c r="AM3" s="1"/>
       <c r="AN3" s="1"/>
       <c r="AO3" s="1"/>
@@ -1528,47 +1504,45 @@
       <c r="AU3" s="1"/>
       <c r="AV3" s="1"/>
       <c r="AW3" s="1"/>
-      <c r="AX3" s="1"/>
+      <c r="AX3" s="8"/>
       <c r="AY3" s="1"/>
-      <c r="AZ3" s="8"/>
-      <c r="BA3" s="1"/>
+      <c r="AZ3" s="1"/>
+      <c r="BA3" s="8"/>
       <c r="BB3" s="1"/>
-      <c r="BC3" s="8"/>
-      <c r="BD3" s="1"/>
-      <c r="BE3" s="4"/>
-      <c r="BF3" s="4"/>
-      <c r="BG3" s="1"/>
+      <c r="BC3" s="4"/>
+      <c r="BD3" s="4"/>
+      <c r="BE3" s="1"/>
+      <c r="BF3" s="1"/>
+      <c r="BG3" s="2"/>
       <c r="BH3" s="1"/>
-      <c r="BI3" s="2"/>
+      <c r="BI3" s="1"/>
       <c r="BJ3" s="1"/>
       <c r="BK3" s="1"/>
-      <c r="BL3" s="1"/>
-      <c r="BM3" s="1"/>
-      <c r="BN3" s="4"/>
-      <c r="BO3" s="4"/>
-      <c r="BP3" s="1"/>
+      <c r="BL3" s="4"/>
+      <c r="BM3" s="4"/>
+      <c r="BN3" s="1"/>
+      <c r="BO3" s="1"/>
+      <c r="BP3" s="4"/>
       <c r="BQ3" s="1"/>
-      <c r="BR3" s="4"/>
+      <c r="BR3" s="1"/>
       <c r="BS3" s="1"/>
-      <c r="BT3" s="1"/>
-      <c r="BU3" s="1"/>
-      <c r="BX3" s="1"/>
-      <c r="BZ3" s="4"/>
-      <c r="CB3" s="2"/>
-      <c r="CC3" s="2"/>
-      <c r="CD3" s="1"/>
+      <c r="BV3" s="1"/>
+      <c r="BX3" s="4"/>
+      <c r="BZ3" s="10"/>
+      <c r="CA3" s="2"/>
+      <c r="CB3" s="1"/>
+      <c r="CC3" s="1"/>
+      <c r="CD3" s="3"/>
       <c r="CE3" s="1"/>
-      <c r="CF3" s="3"/>
-      <c r="CG3" s="1"/>
-      <c r="CH3" s="8"/>
-      <c r="CI3" s="6"/>
-      <c r="CJ3" s="1"/>
-      <c r="CK3" s="1"/>
-      <c r="CM3" s="4"/>
-      <c r="CN3" s="3"/>
-      <c r="CO3" s="1"/>
+      <c r="CF3" s="8"/>
+      <c r="CG3" s="6"/>
+      <c r="CH3" s="1"/>
+      <c r="CI3" s="1"/>
+      <c r="CK3" s="4"/>
+      <c r="CL3" s="3"/>
+      <c r="CM3" s="1"/>
     </row>
-    <row r="4" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
@@ -1582,31 +1556,31 @@
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="1"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="8"/>
       <c r="T4" s="8"/>
-      <c r="U4" s="8"/>
-      <c r="V4" s="1"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="4"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
-      <c r="AA4" s="1"/>
-      <c r="AB4" s="6"/>
-      <c r="AC4" s="6"/>
+      <c r="AA4" s="6"/>
+      <c r="AB4" s="1"/>
+      <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
       <c r="AE4" s="1"/>
       <c r="AF4" s="1"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="1"/>
-      <c r="AI4" s="4"/>
-      <c r="AJ4" s="8"/>
-      <c r="AK4" s="8"/>
-      <c r="AL4" s="4"/>
+      <c r="AG4" s="4"/>
+      <c r="AH4" s="8"/>
+      <c r="AI4" s="8"/>
+      <c r="AJ4" s="4"/>
+      <c r="AK4" s="1"/>
+      <c r="AL4" s="1"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="1"/>
       <c r="AO4" s="1"/>
@@ -1618,47 +1592,45 @@
       <c r="AU4" s="1"/>
       <c r="AV4" s="1"/>
       <c r="AW4" s="1"/>
-      <c r="AX4" s="1"/>
+      <c r="AX4" s="8"/>
       <c r="AY4" s="1"/>
-      <c r="AZ4" s="8"/>
-      <c r="BA4" s="1"/>
+      <c r="AZ4" s="1"/>
+      <c r="BA4" s="8"/>
       <c r="BB4" s="1"/>
-      <c r="BC4" s="8"/>
-      <c r="BD4" s="1"/>
-      <c r="BE4" s="4"/>
-      <c r="BF4" s="4"/>
-      <c r="BG4" s="1"/>
+      <c r="BC4" s="4"/>
+      <c r="BD4" s="4"/>
+      <c r="BE4" s="1"/>
+      <c r="BF4" s="1"/>
+      <c r="BG4" s="2"/>
       <c r="BH4" s="1"/>
-      <c r="BI4" s="2"/>
+      <c r="BI4" s="1"/>
       <c r="BJ4" s="1"/>
       <c r="BK4" s="1"/>
-      <c r="BL4" s="1"/>
-      <c r="BM4" s="1"/>
-      <c r="BN4" s="4"/>
-      <c r="BO4" s="4"/>
-      <c r="BP4" s="1"/>
+      <c r="BL4" s="4"/>
+      <c r="BM4" s="4"/>
+      <c r="BN4" s="1"/>
+      <c r="BO4" s="1"/>
+      <c r="BP4" s="4"/>
       <c r="BQ4" s="1"/>
-      <c r="BR4" s="4"/>
+      <c r="BR4" s="1"/>
       <c r="BS4" s="1"/>
-      <c r="BT4" s="1"/>
-      <c r="BU4" s="1"/>
-      <c r="BX4" s="1"/>
-      <c r="BZ4" s="4"/>
-      <c r="CB4" s="2"/>
-      <c r="CC4" s="2"/>
-      <c r="CD4" s="1"/>
+      <c r="BV4" s="1"/>
+      <c r="BX4" s="4"/>
+      <c r="BZ4" s="2"/>
+      <c r="CA4" s="2"/>
+      <c r="CB4" s="1"/>
+      <c r="CC4" s="1"/>
+      <c r="CD4" s="3"/>
       <c r="CE4" s="1"/>
-      <c r="CF4" s="3"/>
-      <c r="CG4" s="1"/>
-      <c r="CH4" s="8"/>
-      <c r="CI4" s="6"/>
-      <c r="CJ4" s="1"/>
-      <c r="CK4" s="1"/>
-      <c r="CM4" s="4"/>
-      <c r="CN4" s="3"/>
-      <c r="CO4" s="1"/>
+      <c r="CF4" s="8"/>
+      <c r="CG4" s="6"/>
+      <c r="CH4" s="1"/>
+      <c r="CI4" s="1"/>
+      <c r="CK4" s="4"/>
+      <c r="CL4" s="3"/>
+      <c r="CM4" s="1"/>
     </row>
-    <row r="5" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
       <c r="C5" s="3"/>
@@ -1672,31 +1644,31 @@
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="1"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="8"/>
       <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="1"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="4"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
-      <c r="AA5" s="1"/>
-      <c r="AB5" s="6"/>
-      <c r="AC5" s="6"/>
+      <c r="AA5" s="6"/>
+      <c r="AB5" s="1"/>
+      <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
       <c r="AE5" s="1"/>
       <c r="AF5" s="1"/>
-      <c r="AG5" s="1"/>
-      <c r="AH5" s="1"/>
-      <c r="AI5" s="4"/>
-      <c r="AJ5" s="8"/>
-      <c r="AK5" s="8"/>
-      <c r="AL5" s="4"/>
+      <c r="AG5" s="4"/>
+      <c r="AH5" s="8"/>
+      <c r="AI5" s="8"/>
+      <c r="AJ5" s="4"/>
+      <c r="AK5" s="1"/>
+      <c r="AL5" s="1"/>
       <c r="AM5" s="1"/>
       <c r="AN5" s="1"/>
       <c r="AO5" s="1"/>
@@ -1708,47 +1680,45 @@
       <c r="AU5" s="1"/>
       <c r="AV5" s="1"/>
       <c r="AW5" s="1"/>
-      <c r="AX5" s="1"/>
+      <c r="AX5" s="8"/>
       <c r="AY5" s="1"/>
-      <c r="AZ5" s="8"/>
-      <c r="BA5" s="1"/>
+      <c r="AZ5" s="1"/>
+      <c r="BA5" s="8"/>
       <c r="BB5" s="1"/>
-      <c r="BC5" s="8"/>
-      <c r="BD5" s="1"/>
-      <c r="BE5" s="4"/>
-      <c r="BF5" s="4"/>
-      <c r="BG5" s="1"/>
+      <c r="BC5" s="4"/>
+      <c r="BD5" s="4"/>
+      <c r="BE5" s="1"/>
+      <c r="BF5" s="1"/>
+      <c r="BG5" s="2"/>
       <c r="BH5" s="1"/>
-      <c r="BI5" s="2"/>
+      <c r="BI5" s="1"/>
       <c r="BJ5" s="1"/>
       <c r="BK5" s="1"/>
-      <c r="BL5" s="1"/>
-      <c r="BM5" s="1"/>
-      <c r="BN5" s="4"/>
-      <c r="BO5" s="4"/>
-      <c r="BP5" s="1"/>
+      <c r="BL5" s="4"/>
+      <c r="BM5" s="4"/>
+      <c r="BN5" s="1"/>
+      <c r="BO5" s="1"/>
+      <c r="BP5" s="4"/>
       <c r="BQ5" s="1"/>
-      <c r="BR5" s="4"/>
+      <c r="BR5" s="1"/>
       <c r="BS5" s="1"/>
-      <c r="BT5" s="1"/>
-      <c r="BU5" s="1"/>
-      <c r="BX5" s="1"/>
-      <c r="BZ5" s="4"/>
-      <c r="CB5" s="2"/>
-      <c r="CC5" s="2"/>
-      <c r="CD5" s="1"/>
+      <c r="BV5" s="1"/>
+      <c r="BX5" s="4"/>
+      <c r="BZ5" s="2"/>
+      <c r="CA5" s="2"/>
+      <c r="CB5" s="1"/>
+      <c r="CC5" s="1"/>
+      <c r="CD5" s="3"/>
       <c r="CE5" s="1"/>
-      <c r="CF5" s="3"/>
-      <c r="CG5" s="1"/>
-      <c r="CH5" s="8"/>
-      <c r="CI5" s="6"/>
-      <c r="CJ5" s="1"/>
-      <c r="CK5" s="1"/>
-      <c r="CM5" s="4"/>
-      <c r="CN5" s="3"/>
-      <c r="CO5" s="1"/>
+      <c r="CF5" s="8"/>
+      <c r="CG5" s="6"/>
+      <c r="CH5" s="1"/>
+      <c r="CI5" s="1"/>
+      <c r="CK5" s="4"/>
+      <c r="CL5" s="3"/>
+      <c r="CM5" s="1"/>
     </row>
-    <row r="6" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
@@ -1762,31 +1732,31 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="1"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="8"/>
       <c r="T6" s="8"/>
-      <c r="U6" s="8"/>
-      <c r="V6" s="1"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="4"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="6"/>
-      <c r="AC6" s="4"/>
+      <c r="AA6" s="6"/>
+      <c r="AB6" s="1"/>
+      <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
-      <c r="AG6" s="1"/>
-      <c r="AH6" s="1"/>
-      <c r="AI6" s="4"/>
-      <c r="AJ6" s="8"/>
-      <c r="AK6" s="8"/>
-      <c r="AL6" s="4"/>
+      <c r="AG6" s="4"/>
+      <c r="AH6" s="8"/>
+      <c r="AI6" s="8"/>
+      <c r="AJ6" s="4"/>
+      <c r="AK6" s="1"/>
+      <c r="AL6" s="1"/>
       <c r="AM6" s="1"/>
       <c r="AN6" s="1"/>
       <c r="AO6" s="1"/>
@@ -1798,46 +1768,44 @@
       <c r="AU6" s="1"/>
       <c r="AV6" s="1"/>
       <c r="AW6" s="1"/>
-      <c r="AX6" s="1"/>
+      <c r="AX6" s="8"/>
       <c r="AY6" s="1"/>
-      <c r="AZ6" s="8"/>
-      <c r="BA6" s="1"/>
+      <c r="AZ6" s="1"/>
+      <c r="BA6" s="8"/>
       <c r="BB6" s="1"/>
-      <c r="BC6" s="8"/>
-      <c r="BD6" s="1"/>
-      <c r="BE6" s="4"/>
-      <c r="BF6" s="4"/>
-      <c r="BG6" s="1"/>
+      <c r="BC6" s="4"/>
+      <c r="BD6" s="4"/>
+      <c r="BE6" s="1"/>
+      <c r="BF6" s="1"/>
+      <c r="BG6" s="2"/>
       <c r="BH6" s="1"/>
-      <c r="BI6" s="2"/>
+      <c r="BI6" s="1"/>
       <c r="BJ6" s="1"/>
       <c r="BK6" s="1"/>
-      <c r="BL6" s="1"/>
-      <c r="BM6" s="1"/>
-      <c r="BN6" s="4"/>
-      <c r="BO6" s="4"/>
-      <c r="BP6" s="1"/>
+      <c r="BL6" s="4"/>
+      <c r="BM6" s="4"/>
+      <c r="BN6" s="1"/>
+      <c r="BO6" s="1"/>
       <c r="BQ6" s="1"/>
+      <c r="BR6" s="1"/>
       <c r="BS6" s="1"/>
-      <c r="BT6" s="1"/>
-      <c r="BU6" s="1"/>
-      <c r="BX6" s="1"/>
-      <c r="BZ6" s="4"/>
-      <c r="CB6" s="2"/>
-      <c r="CC6" s="2"/>
-      <c r="CD6" s="1"/>
+      <c r="BV6" s="1"/>
+      <c r="BX6" s="4"/>
+      <c r="BZ6" s="2"/>
+      <c r="CA6" s="2"/>
+      <c r="CB6" s="1"/>
+      <c r="CC6" s="1"/>
+      <c r="CD6" s="3"/>
       <c r="CE6" s="1"/>
-      <c r="CF6" s="3"/>
-      <c r="CG6" s="1"/>
-      <c r="CH6" s="8"/>
-      <c r="CI6" s="6"/>
-      <c r="CJ6" s="1"/>
-      <c r="CK6" s="1"/>
-      <c r="CM6" s="4"/>
-      <c r="CN6" s="3"/>
-      <c r="CO6" s="1"/>
+      <c r="CF6" s="8"/>
+      <c r="CG6" s="6"/>
+      <c r="CH6" s="1"/>
+      <c r="CI6" s="1"/>
+      <c r="CK6" s="4"/>
+      <c r="CL6" s="3"/>
+      <c r="CM6" s="1"/>
     </row>
-    <row r="7" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>
@@ -1851,31 +1819,31 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="1"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="8"/>
       <c r="T7" s="8"/>
-      <c r="U7" s="8"/>
-      <c r="V7" s="1"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="4"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="4"/>
+      <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="6"/>
-      <c r="AC7" s="4"/>
+      <c r="AA7" s="6"/>
+      <c r="AB7" s="1"/>
+      <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="1"/>
-      <c r="AI7" s="4"/>
-      <c r="AJ7" s="8"/>
-      <c r="AK7" s="8"/>
-      <c r="AL7" s="4"/>
+      <c r="AG7" s="4"/>
+      <c r="AH7" s="8"/>
+      <c r="AI7" s="8"/>
+      <c r="AJ7" s="4"/>
+      <c r="AK7" s="1"/>
+      <c r="AL7" s="1"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="1"/>
       <c r="AO7" s="1"/>
@@ -1887,46 +1855,44 @@
       <c r="AU7" s="1"/>
       <c r="AV7" s="1"/>
       <c r="AW7" s="1"/>
-      <c r="AX7" s="1"/>
+      <c r="AX7" s="8"/>
       <c r="AY7" s="1"/>
-      <c r="AZ7" s="8"/>
-      <c r="BA7" s="1"/>
+      <c r="AZ7" s="1"/>
+      <c r="BA7" s="8"/>
       <c r="BB7" s="1"/>
-      <c r="BC7" s="8"/>
-      <c r="BD7" s="1"/>
-      <c r="BE7" s="4"/>
-      <c r="BF7" s="4"/>
-      <c r="BG7" s="1"/>
+      <c r="BC7" s="4"/>
+      <c r="BD7" s="4"/>
+      <c r="BE7" s="1"/>
+      <c r="BF7" s="1"/>
+      <c r="BG7" s="2"/>
       <c r="BH7" s="1"/>
-      <c r="BI7" s="2"/>
+      <c r="BI7" s="1"/>
       <c r="BJ7" s="1"/>
       <c r="BK7" s="1"/>
-      <c r="BL7" s="1"/>
-      <c r="BM7" s="1"/>
-      <c r="BN7" s="4"/>
-      <c r="BO7" s="4"/>
-      <c r="BP7" s="1"/>
+      <c r="BL7" s="4"/>
+      <c r="BM7" s="4"/>
+      <c r="BN7" s="1"/>
+      <c r="BO7" s="1"/>
       <c r="BQ7" s="1"/>
+      <c r="BR7" s="1"/>
       <c r="BS7" s="1"/>
-      <c r="BT7" s="1"/>
-      <c r="BU7" s="1"/>
-      <c r="BX7" s="1"/>
-      <c r="BZ7" s="4"/>
-      <c r="CB7" s="2"/>
-      <c r="CC7" s="2"/>
-      <c r="CD7" s="1"/>
+      <c r="BV7" s="1"/>
+      <c r="BX7" s="4"/>
+      <c r="BZ7" s="2"/>
+      <c r="CA7" s="2"/>
+      <c r="CB7" s="1"/>
+      <c r="CC7" s="1"/>
+      <c r="CD7" s="3"/>
       <c r="CE7" s="1"/>
-      <c r="CF7" s="3"/>
-      <c r="CG7" s="1"/>
-      <c r="CH7" s="8"/>
-      <c r="CI7" s="6"/>
-      <c r="CJ7" s="1"/>
-      <c r="CK7" s="1"/>
-      <c r="CM7" s="4"/>
-      <c r="CN7" s="3"/>
-      <c r="CO7" s="1"/>
+      <c r="CF7" s="8"/>
+      <c r="CG7" s="6"/>
+      <c r="CH7" s="1"/>
+      <c r="CI7" s="1"/>
+      <c r="CK7" s="4"/>
+      <c r="CL7" s="3"/>
+      <c r="CM7" s="1"/>
     </row>
-    <row r="8" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="2"/>
       <c r="C8" s="3"/>
@@ -1940,31 +1906,31 @@
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="1"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="8"/>
       <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
-      <c r="V8" s="1"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="4"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="4"/>
+      <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="6"/>
-      <c r="AC8" s="4"/>
+      <c r="AA8" s="6"/>
+      <c r="AB8" s="1"/>
+      <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
       <c r="AE8" s="1"/>
       <c r="AF8" s="1"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="1"/>
-      <c r="AI8" s="4"/>
-      <c r="AJ8" s="8"/>
-      <c r="AK8" s="8"/>
-      <c r="AL8" s="4"/>
+      <c r="AG8" s="4"/>
+      <c r="AH8" s="8"/>
+      <c r="AI8" s="8"/>
+      <c r="AJ8" s="4"/>
+      <c r="AK8" s="1"/>
+      <c r="AL8" s="1"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="1"/>
       <c r="AO8" s="1"/>
@@ -1976,46 +1942,44 @@
       <c r="AU8" s="1"/>
       <c r="AV8" s="1"/>
       <c r="AW8" s="1"/>
-      <c r="AX8" s="1"/>
+      <c r="AX8" s="8"/>
       <c r="AY8" s="1"/>
-      <c r="AZ8" s="8"/>
-      <c r="BA8" s="1"/>
+      <c r="AZ8" s="1"/>
+      <c r="BA8" s="8"/>
       <c r="BB8" s="1"/>
-      <c r="BC8" s="8"/>
-      <c r="BD8" s="1"/>
-      <c r="BE8" s="4"/>
-      <c r="BF8" s="4"/>
-      <c r="BG8" s="1"/>
+      <c r="BC8" s="4"/>
+      <c r="BD8" s="4"/>
+      <c r="BE8" s="1"/>
+      <c r="BF8" s="1"/>
+      <c r="BG8" s="2"/>
       <c r="BH8" s="1"/>
-      <c r="BI8" s="2"/>
+      <c r="BI8" s="1"/>
       <c r="BJ8" s="1"/>
       <c r="BK8" s="1"/>
-      <c r="BL8" s="1"/>
-      <c r="BM8" s="1"/>
-      <c r="BN8" s="4"/>
-      <c r="BO8" s="4"/>
-      <c r="BP8" s="1"/>
+      <c r="BL8" s="4"/>
+      <c r="BM8" s="4"/>
+      <c r="BN8" s="1"/>
+      <c r="BO8" s="1"/>
       <c r="BQ8" s="1"/>
+      <c r="BR8" s="1"/>
       <c r="BS8" s="1"/>
-      <c r="BT8" s="1"/>
-      <c r="BU8" s="1"/>
-      <c r="BX8" s="1"/>
-      <c r="BZ8" s="4"/>
-      <c r="CB8" s="2"/>
-      <c r="CC8" s="2"/>
-      <c r="CD8" s="1"/>
+      <c r="BV8" s="1"/>
+      <c r="BX8" s="4"/>
+      <c r="BZ8" s="2"/>
+      <c r="CA8" s="2"/>
+      <c r="CB8" s="1"/>
+      <c r="CC8" s="1"/>
+      <c r="CD8" s="3"/>
       <c r="CE8" s="1"/>
-      <c r="CF8" s="3"/>
-      <c r="CG8" s="1"/>
-      <c r="CH8" s="8"/>
-      <c r="CI8" s="6"/>
-      <c r="CJ8" s="1"/>
-      <c r="CK8" s="1"/>
-      <c r="CM8" s="4"/>
-      <c r="CN8" s="3"/>
-      <c r="CO8" s="1"/>
+      <c r="CF8" s="8"/>
+      <c r="CG8" s="6"/>
+      <c r="CH8" s="1"/>
+      <c r="CI8" s="1"/>
+      <c r="CK8" s="4"/>
+      <c r="CL8" s="3"/>
+      <c r="CM8" s="1"/>
     </row>
-    <row r="9" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="2"/>
       <c r="C9" s="3"/>
@@ -2029,31 +1993,31 @@
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="1"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="8"/>
       <c r="T9" s="8"/>
-      <c r="U9" s="8"/>
-      <c r="V9" s="1"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="4"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="4"/>
+      <c r="X9" s="1"/>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
-      <c r="AA9" s="1"/>
-      <c r="AB9" s="6"/>
-      <c r="AC9" s="4"/>
+      <c r="AA9" s="6"/>
+      <c r="AB9" s="1"/>
+      <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
       <c r="AE9" s="1"/>
       <c r="AF9" s="1"/>
-      <c r="AG9" s="1"/>
-      <c r="AH9" s="1"/>
-      <c r="AI9" s="4"/>
-      <c r="AJ9" s="8"/>
-      <c r="AK9" s="8"/>
-      <c r="AL9" s="4"/>
+      <c r="AG9" s="4"/>
+      <c r="AH9" s="8"/>
+      <c r="AI9" s="8"/>
+      <c r="AJ9" s="4"/>
+      <c r="AK9" s="1"/>
+      <c r="AL9" s="1"/>
       <c r="AM9" s="1"/>
       <c r="AN9" s="1"/>
       <c r="AO9" s="1"/>
@@ -2065,46 +2029,44 @@
       <c r="AU9" s="1"/>
       <c r="AV9" s="1"/>
       <c r="AW9" s="1"/>
-      <c r="AX9" s="1"/>
+      <c r="AX9" s="8"/>
       <c r="AY9" s="1"/>
-      <c r="AZ9" s="8"/>
-      <c r="BA9" s="1"/>
+      <c r="AZ9" s="1"/>
+      <c r="BA9" s="8"/>
       <c r="BB9" s="1"/>
-      <c r="BC9" s="8"/>
-      <c r="BD9" s="1"/>
-      <c r="BE9" s="4"/>
-      <c r="BF9" s="4"/>
-      <c r="BG9" s="1"/>
+      <c r="BC9" s="4"/>
+      <c r="BD9" s="4"/>
+      <c r="BE9" s="1"/>
+      <c r="BF9" s="1"/>
+      <c r="BG9" s="2"/>
       <c r="BH9" s="1"/>
-      <c r="BI9" s="2"/>
+      <c r="BI9" s="1"/>
       <c r="BJ9" s="1"/>
       <c r="BK9" s="1"/>
-      <c r="BL9" s="1"/>
-      <c r="BM9" s="1"/>
-      <c r="BN9" s="4"/>
-      <c r="BO9" s="4"/>
-      <c r="BP9" s="1"/>
+      <c r="BL9" s="4"/>
+      <c r="BM9" s="4"/>
+      <c r="BN9" s="1"/>
+      <c r="BO9" s="1"/>
       <c r="BQ9" s="1"/>
+      <c r="BR9" s="1"/>
       <c r="BS9" s="1"/>
-      <c r="BT9" s="1"/>
-      <c r="BU9" s="1"/>
-      <c r="BX9" s="1"/>
-      <c r="BZ9" s="4"/>
-      <c r="CB9" s="2"/>
-      <c r="CC9" s="2"/>
-      <c r="CD9" s="1"/>
+      <c r="BV9" s="1"/>
+      <c r="BX9" s="4"/>
+      <c r="BZ9" s="2"/>
+      <c r="CA9" s="2"/>
+      <c r="CB9" s="1"/>
+      <c r="CC9" s="1"/>
+      <c r="CD9" s="3"/>
       <c r="CE9" s="1"/>
-      <c r="CF9" s="3"/>
-      <c r="CG9" s="1"/>
-      <c r="CH9" s="8"/>
-      <c r="CI9" s="6"/>
-      <c r="CJ9" s="1"/>
-      <c r="CK9" s="1"/>
-      <c r="CM9" s="4"/>
-      <c r="CN9" s="3"/>
-      <c r="CO9" s="1"/>
+      <c r="CF9" s="8"/>
+      <c r="CG9" s="6"/>
+      <c r="CH9" s="1"/>
+      <c r="CI9" s="1"/>
+      <c r="CK9" s="4"/>
+      <c r="CL9" s="3"/>
+      <c r="CM9" s="1"/>
     </row>
-    <row r="10" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="2"/>
       <c r="C10" s="3"/>
@@ -2118,31 +2080,31 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="1"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="8"/>
       <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="1"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="4"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="4"/>
+      <c r="X10" s="1"/>
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
-      <c r="AA10" s="1"/>
-      <c r="AB10" s="6"/>
-      <c r="AC10" s="6"/>
+      <c r="AA10" s="6"/>
+      <c r="AB10" s="1"/>
+      <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
       <c r="AE10" s="1"/>
       <c r="AF10" s="1"/>
-      <c r="AG10" s="1"/>
-      <c r="AH10" s="1"/>
-      <c r="AI10" s="4"/>
-      <c r="AJ10" s="8"/>
-      <c r="AK10" s="8"/>
-      <c r="AL10" s="4"/>
+      <c r="AG10" s="4"/>
+      <c r="AH10" s="8"/>
+      <c r="AI10" s="8"/>
+      <c r="AJ10" s="4"/>
+      <c r="AK10" s="1"/>
+      <c r="AL10" s="1"/>
       <c r="AM10" s="1"/>
       <c r="AN10" s="1"/>
       <c r="AO10" s="1"/>
@@ -2154,47 +2116,45 @@
       <c r="AU10" s="1"/>
       <c r="AV10" s="1"/>
       <c r="AW10" s="1"/>
-      <c r="AX10" s="1"/>
+      <c r="AX10" s="8"/>
       <c r="AY10" s="1"/>
-      <c r="AZ10" s="8"/>
-      <c r="BA10" s="1"/>
+      <c r="AZ10" s="1"/>
+      <c r="BA10" s="8"/>
       <c r="BB10" s="1"/>
-      <c r="BC10" s="8"/>
-      <c r="BD10" s="1"/>
-      <c r="BE10" s="4"/>
-      <c r="BF10" s="4"/>
-      <c r="BG10" s="1"/>
+      <c r="BC10" s="4"/>
+      <c r="BD10" s="4"/>
+      <c r="BE10" s="1"/>
+      <c r="BF10" s="1"/>
+      <c r="BG10" s="2"/>
       <c r="BH10" s="1"/>
-      <c r="BI10" s="2"/>
+      <c r="BI10" s="1"/>
       <c r="BJ10" s="1"/>
       <c r="BK10" s="1"/>
-      <c r="BL10" s="1"/>
-      <c r="BM10" s="1"/>
-      <c r="BN10" s="4"/>
-      <c r="BO10" s="4"/>
-      <c r="BP10" s="1"/>
+      <c r="BL10" s="4"/>
+      <c r="BM10" s="4"/>
+      <c r="BN10" s="1"/>
+      <c r="BO10" s="1"/>
+      <c r="BP10" s="4"/>
       <c r="BQ10" s="1"/>
-      <c r="BR10" s="4"/>
+      <c r="BR10" s="1"/>
       <c r="BS10" s="1"/>
-      <c r="BT10" s="1"/>
-      <c r="BU10" s="1"/>
-      <c r="BX10" s="1"/>
-      <c r="BZ10" s="4"/>
-      <c r="CB10" s="2"/>
-      <c r="CC10" s="2"/>
-      <c r="CD10" s="1"/>
+      <c r="BV10" s="1"/>
+      <c r="BX10" s="4"/>
+      <c r="BZ10" s="2"/>
+      <c r="CA10" s="2"/>
+      <c r="CB10" s="1"/>
+      <c r="CC10" s="1"/>
+      <c r="CD10" s="3"/>
       <c r="CE10" s="1"/>
-      <c r="CF10" s="3"/>
-      <c r="CG10" s="1"/>
-      <c r="CH10" s="8"/>
-      <c r="CI10" s="4"/>
-      <c r="CJ10" s="1"/>
-      <c r="CK10" s="1"/>
-      <c r="CM10" s="4"/>
-      <c r="CN10" s="3"/>
-      <c r="CO10" s="1"/>
+      <c r="CF10" s="8"/>
+      <c r="CG10" s="4"/>
+      <c r="CH10" s="1"/>
+      <c r="CI10" s="1"/>
+      <c r="CK10" s="4"/>
+      <c r="CL10" s="3"/>
+      <c r="CM10" s="1"/>
     </row>
-    <row r="11" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="2"/>
       <c r="C11" s="3"/>
@@ -2208,31 +2168,31 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="1"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="8"/>
       <c r="T11" s="8"/>
-      <c r="U11" s="8"/>
-      <c r="V11" s="1"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="4"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="4"/>
+      <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
-      <c r="AA11" s="1"/>
-      <c r="AB11" s="6"/>
-      <c r="AC11" s="6"/>
+      <c r="AA11" s="6"/>
+      <c r="AB11" s="1"/>
+      <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
       <c r="AE11" s="1"/>
       <c r="AF11" s="1"/>
-      <c r="AG11" s="1"/>
-      <c r="AH11" s="1"/>
-      <c r="AI11" s="4"/>
-      <c r="AJ11" s="8"/>
-      <c r="AK11" s="8"/>
-      <c r="AL11" s="4"/>
+      <c r="AG11" s="4"/>
+      <c r="AH11" s="8"/>
+      <c r="AI11" s="8"/>
+      <c r="AJ11" s="4"/>
+      <c r="AK11" s="1"/>
+      <c r="AL11" s="1"/>
       <c r="AM11" s="1"/>
       <c r="AN11" s="1"/>
       <c r="AO11" s="1"/>
@@ -2244,47 +2204,45 @@
       <c r="AU11" s="1"/>
       <c r="AV11" s="1"/>
       <c r="AW11" s="1"/>
-      <c r="AX11" s="1"/>
+      <c r="AX11" s="8"/>
       <c r="AY11" s="1"/>
-      <c r="AZ11" s="8"/>
-      <c r="BA11" s="1"/>
+      <c r="AZ11" s="1"/>
+      <c r="BA11" s="8"/>
       <c r="BB11" s="1"/>
-      <c r="BC11" s="8"/>
-      <c r="BD11" s="1"/>
-      <c r="BE11" s="4"/>
-      <c r="BF11" s="4"/>
-      <c r="BG11" s="1"/>
+      <c r="BC11" s="4"/>
+      <c r="BD11" s="4"/>
+      <c r="BE11" s="1"/>
+      <c r="BF11" s="1"/>
+      <c r="BG11" s="2"/>
       <c r="BH11" s="1"/>
-      <c r="BI11" s="2"/>
+      <c r="BI11" s="1"/>
       <c r="BJ11" s="1"/>
       <c r="BK11" s="1"/>
-      <c r="BL11" s="1"/>
-      <c r="BM11" s="1"/>
-      <c r="BN11" s="4"/>
-      <c r="BO11" s="4"/>
-      <c r="BP11" s="1"/>
+      <c r="BL11" s="4"/>
+      <c r="BM11" s="4"/>
+      <c r="BN11" s="1"/>
+      <c r="BO11" s="1"/>
+      <c r="BP11" s="4"/>
       <c r="BQ11" s="1"/>
-      <c r="BR11" s="4"/>
+      <c r="BR11" s="1"/>
       <c r="BS11" s="1"/>
-      <c r="BT11" s="1"/>
-      <c r="BU11" s="1"/>
-      <c r="BX11" s="1"/>
-      <c r="BZ11" s="4"/>
-      <c r="CB11" s="2"/>
-      <c r="CC11" s="2"/>
-      <c r="CD11" s="1"/>
+      <c r="BV11" s="1"/>
+      <c r="BX11" s="4"/>
+      <c r="BZ11" s="2"/>
+      <c r="CA11" s="2"/>
+      <c r="CB11" s="1"/>
+      <c r="CC11" s="1"/>
+      <c r="CD11" s="3"/>
       <c r="CE11" s="1"/>
-      <c r="CF11" s="3"/>
-      <c r="CG11" s="1"/>
-      <c r="CH11" s="8"/>
-      <c r="CI11" s="4"/>
-      <c r="CJ11" s="1"/>
-      <c r="CK11" s="1"/>
-      <c r="CM11" s="4"/>
-      <c r="CN11" s="3"/>
-      <c r="CO11" s="1"/>
+      <c r="CF11" s="8"/>
+      <c r="CG11" s="4"/>
+      <c r="CH11" s="1"/>
+      <c r="CI11" s="1"/>
+      <c r="CK11" s="4"/>
+      <c r="CL11" s="3"/>
+      <c r="CM11" s="1"/>
     </row>
-    <row r="12" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="2"/>
       <c r="C12" s="3"/>
@@ -2298,31 +2256,31 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="5"/>
-      <c r="S12" s="1"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="1"/>
+      <c r="S12" s="8"/>
       <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="1"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="4"/>
+      <c r="U12" s="1"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="4"/>
+      <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
-      <c r="AA12" s="1"/>
-      <c r="AB12" s="6"/>
-      <c r="AC12" s="6"/>
+      <c r="AA12" s="6"/>
+      <c r="AB12" s="1"/>
+      <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
       <c r="AE12" s="1"/>
       <c r="AF12" s="1"/>
-      <c r="AG12" s="1"/>
-      <c r="AH12" s="1"/>
-      <c r="AI12" s="4"/>
-      <c r="AJ12" s="8"/>
-      <c r="AK12" s="8"/>
-      <c r="AL12" s="4"/>
+      <c r="AG12" s="4"/>
+      <c r="AH12" s="8"/>
+      <c r="AI12" s="8"/>
+      <c r="AJ12" s="4"/>
+      <c r="AK12" s="1"/>
+      <c r="AL12" s="1"/>
       <c r="AM12" s="1"/>
       <c r="AN12" s="1"/>
       <c r="AO12" s="1"/>
@@ -2334,47 +2292,45 @@
       <c r="AU12" s="1"/>
       <c r="AV12" s="1"/>
       <c r="AW12" s="1"/>
-      <c r="AX12" s="1"/>
+      <c r="AX12" s="8"/>
       <c r="AY12" s="1"/>
-      <c r="AZ12" s="8"/>
-      <c r="BA12" s="1"/>
+      <c r="AZ12" s="1"/>
+      <c r="BA12" s="8"/>
       <c r="BB12" s="1"/>
-      <c r="BC12" s="8"/>
-      <c r="BD12" s="1"/>
-      <c r="BE12" s="4"/>
-      <c r="BF12" s="4"/>
-      <c r="BG12" s="1"/>
+      <c r="BC12" s="4"/>
+      <c r="BD12" s="4"/>
+      <c r="BE12" s="1"/>
+      <c r="BF12" s="1"/>
+      <c r="BG12" s="2"/>
       <c r="BH12" s="1"/>
-      <c r="BI12" s="2"/>
+      <c r="BI12" s="1"/>
       <c r="BJ12" s="1"/>
       <c r="BK12" s="1"/>
-      <c r="BL12" s="1"/>
-      <c r="BM12" s="1"/>
-      <c r="BN12" s="4"/>
-      <c r="BO12" s="4"/>
-      <c r="BP12" s="1"/>
+      <c r="BL12" s="4"/>
+      <c r="BM12" s="4"/>
+      <c r="BN12" s="1"/>
+      <c r="BO12" s="1"/>
+      <c r="BP12" s="4"/>
       <c r="BQ12" s="1"/>
-      <c r="BR12" s="4"/>
+      <c r="BR12" s="1"/>
       <c r="BS12" s="1"/>
-      <c r="BT12" s="1"/>
-      <c r="BU12" s="1"/>
-      <c r="BX12" s="1"/>
-      <c r="BZ12" s="4"/>
-      <c r="CB12" s="2"/>
-      <c r="CC12" s="2"/>
-      <c r="CD12" s="1"/>
+      <c r="BV12" s="1"/>
+      <c r="BX12" s="4"/>
+      <c r="BZ12" s="2"/>
+      <c r="CA12" s="2"/>
+      <c r="CB12" s="1"/>
+      <c r="CC12" s="1"/>
+      <c r="CD12" s="3"/>
       <c r="CE12" s="1"/>
-      <c r="CF12" s="3"/>
-      <c r="CG12" s="1"/>
-      <c r="CH12" s="8"/>
-      <c r="CI12" s="4"/>
-      <c r="CJ12" s="1"/>
-      <c r="CK12" s="1"/>
-      <c r="CM12" s="4"/>
-      <c r="CN12" s="3"/>
-      <c r="CO12" s="1"/>
+      <c r="CF12" s="8"/>
+      <c r="CG12" s="4"/>
+      <c r="CH12" s="1"/>
+      <c r="CI12" s="1"/>
+      <c r="CK12" s="4"/>
+      <c r="CL12" s="3"/>
+      <c r="CM12" s="1"/>
     </row>
-    <row r="13" spans="1:97" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:95" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="2"/>
       <c r="C13" s="3"/>
@@ -2388,31 +2344,31 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="1"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="1"/>
+      <c r="S13" s="8"/>
       <c r="T13" s="8"/>
-      <c r="U13" s="8"/>
-      <c r="V13" s="1"/>
-      <c r="W13" s="3"/>
-      <c r="X13" s="4"/>
+      <c r="U13" s="1"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="4"/>
+      <c r="X13" s="1"/>
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
-      <c r="AA13" s="1"/>
-      <c r="AB13" s="6"/>
-      <c r="AC13" s="6"/>
+      <c r="AA13" s="6"/>
+      <c r="AB13" s="1"/>
+      <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
       <c r="AE13" s="1"/>
       <c r="AF13" s="1"/>
-      <c r="AG13" s="1"/>
-      <c r="AH13" s="1"/>
-      <c r="AI13" s="4"/>
-      <c r="AJ13" s="8"/>
-      <c r="AK13" s="8"/>
-      <c r="AL13" s="4"/>
+      <c r="AG13" s="4"/>
+      <c r="AH13" s="8"/>
+      <c r="AI13" s="8"/>
+      <c r="AJ13" s="4"/>
+      <c r="AK13" s="1"/>
+      <c r="AL13" s="1"/>
       <c r="AM13" s="1"/>
       <c r="AN13" s="1"/>
       <c r="AO13" s="1"/>
@@ -2424,45 +2380,43 @@
       <c r="AU13" s="1"/>
       <c r="AV13" s="1"/>
       <c r="AW13" s="1"/>
-      <c r="AX13" s="1"/>
+      <c r="AX13" s="8"/>
       <c r="AY13" s="1"/>
-      <c r="AZ13" s="8"/>
-      <c r="BA13" s="1"/>
+      <c r="AZ13" s="1"/>
+      <c r="BA13" s="8"/>
       <c r="BB13" s="1"/>
-      <c r="BC13" s="8"/>
-      <c r="BD13" s="1"/>
-      <c r="BE13" s="4"/>
-      <c r="BF13" s="4"/>
-      <c r="BG13" s="1"/>
+      <c r="BC13" s="4"/>
+      <c r="BD13" s="4"/>
+      <c r="BE13" s="1"/>
+      <c r="BF13" s="1"/>
+      <c r="BG13" s="2"/>
       <c r="BH13" s="1"/>
-      <c r="BI13" s="2"/>
+      <c r="BI13" s="1"/>
       <c r="BJ13" s="1"/>
       <c r="BK13" s="1"/>
-      <c r="BL13" s="1"/>
-      <c r="BM13" s="1"/>
-      <c r="BN13" s="4"/>
-      <c r="BO13" s="4"/>
-      <c r="BP13" s="1"/>
+      <c r="BL13" s="4"/>
+      <c r="BM13" s="4"/>
+      <c r="BN13" s="1"/>
+      <c r="BO13" s="1"/>
+      <c r="BP13" s="4"/>
       <c r="BQ13" s="1"/>
-      <c r="BR13" s="4"/>
+      <c r="BR13" s="1"/>
       <c r="BS13" s="1"/>
-      <c r="BT13" s="1"/>
-      <c r="BU13" s="1"/>
-      <c r="BX13" s="1"/>
-      <c r="BZ13" s="4"/>
-      <c r="CB13" s="2"/>
-      <c r="CC13" s="2"/>
-      <c r="CD13" s="1"/>
+      <c r="BV13" s="1"/>
+      <c r="BX13" s="4"/>
+      <c r="BZ13" s="2"/>
+      <c r="CA13" s="2"/>
+      <c r="CB13" s="1"/>
+      <c r="CC13" s="1"/>
+      <c r="CD13" s="3"/>
       <c r="CE13" s="1"/>
-      <c r="CF13" s="3"/>
-      <c r="CG13" s="1"/>
-      <c r="CH13" s="8"/>
-      <c r="CI13" s="4"/>
-      <c r="CJ13" s="1"/>
-      <c r="CK13" s="1"/>
-      <c r="CM13" s="4"/>
-      <c r="CN13" s="3"/>
-      <c r="CO13" s="1"/>
+      <c r="CF13" s="8"/>
+      <c r="CG13" s="4"/>
+      <c r="CH13" s="1"/>
+      <c r="CI13" s="1"/>
+      <c r="CK13" s="4"/>
+      <c r="CL13" s="3"/>
+      <c r="CM13" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>